<commit_message>
Corriger le style secondaire de Leona et de Nami.
Leona et Nami ont Counter-engage en secondaire. Le CSV et l'Excel portent la même correction.

Co-authored-by: LeCoonEtSaBande <LeCoonEtSaBande@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Catalogue_champions_LoL.xlsx
+++ b/Catalogue_champions_LoL.xlsx
@@ -3448,7 +3448,11 @@
           <t>Engage</t>
         </is>
       </c>
-      <c r="C74" s="3" t="n"/>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Counter-engage</t>
+        </is>
+      </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
           <t>HP+</t>
@@ -4077,7 +4081,7 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Engage</t>
+          <t>Counter-engage</t>
         </is>
       </c>
       <c r="D91" s="3" t="n"/>

</xml_diff>